<commit_message>
Update course plans and educational programs with quality notes and corrections
- Increased quality notes for several course plans, including GJP37V, GPR256, PR1017, PR1024, PR2003, PR2004, ASS28X, GSS2GP, GSS35H, GTY3J5, GTY3J6, GTY3J7, TY1069, TY1073, TY2004, TY2007, TY2008.
- Added references to confirmed discontinued courses in prerequisites across multiple course plans.
- Corrected discrepancies in program course names and linked them to their respective course codes in educational plans LG79A, LGGYA, LLL6A, and LLP6A.
- Ensured consistency in phrasing and formatting throughout the course plans.
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/02 IHV/Analys/Förkunskapskrav.xlsx
+++ b/vault-dalarna-university/02 IHV/Analys/Förkunskapskrav.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Förkunskapskrav" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Förkunskapskrav'!$A$1:$H$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Förkunskapskrav'!$A$1:$H$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -562,41 +562,49 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>IH2001</t>
+          <t>GSA2AF</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>IDA</t>
+          <t>SAA</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2011-01-26</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr"/>
+          <t>2019-08-29</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2023-09-13</t>
+        </is>
+      </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Refererar troligen nedlagd kurs</t>
+          <t>Refererar bekräftat nedlagd kurs</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Refererad kurs hittas ej i vaulten (troligen nedlagd): 'Idrott 2'</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr"/>
+          <t>`Organisation`</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>`FEB021` (nedlagd 2008-03-18); förkunskap nämner nedlagd kurs</t>
+        </is>
+      </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IH2001</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA2AF</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>GSA2AF</t>
+          <t>GSA2BV</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -606,12 +614,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2019-08-29</t>
+          <t>2019-10-29</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2023-09-13</t>
+          <t>2023-01-19</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -631,14 +639,14 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA2AF</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA2BV</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>GSA2BV</t>
+          <t>GSA2E4</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -648,14 +656,10 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2019-10-29</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>2023-01-19</t>
-        </is>
-      </c>
+          <t>2020-02-13</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
           <t>Refererar bekräftat nedlagd kurs</t>
@@ -673,14 +677,14 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA2BV</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA2E4</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>GSA2E4</t>
+          <t>GSA2E5</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -711,14 +715,14 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA2E4</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA2E5</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>GSA2E5</t>
+          <t>GSA2SD</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -728,7 +732,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2020-02-13</t>
+          <t>2021-12-08</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
@@ -749,14 +753,14 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA2E5</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA2SD</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>GSA2SD</t>
+          <t>GSA2SE</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -787,14 +791,14 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA2SD</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA2SE</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>GSA2SE</t>
+          <t>GSA3FK</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -804,7 +808,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2021-12-08</t>
+          <t>2025-03-07</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
@@ -825,50 +829,12 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA2SE</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>GSA3FK</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>SAA</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>2025-03-07</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>Refererar bekräftat nedlagd kurs</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>`Organisation`</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>`FEB021` (nedlagd 2008-03-18); förkunskap nämner nedlagd kurs</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA3FK</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H11"/>
+  <autoFilter ref="A1:H10"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId2"/>
@@ -888,8 +854,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A10" r:id="rId17"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A11" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId20"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>